<commit_message>
Versión 2.0: fuente Abadi, mayúsculas, portada y ayuda en cada Excel, catálogos editables, conciliación rediseñada, 14 tableros con gráficas, 6 políticas y procedimientos en Word, portadas de venta rediseñadas y por producto
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/ejemplos/1_Contabilidad_y_Finanzas/03_Flujo_de_Efectivo_Anual_EJEMPLO.xlsx
+++ b/ejemplos/1_Contabilidad_y_Finanzas/03_Flujo_de_Efectivo_Anual_EJEMPLO.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formato" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PORTADA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORMATO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMEN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYUDA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,92 +31,145 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <i val="1"/>
       <color rgb="005B6B78"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <i val="1"/>
       <color rgb="00A6A6A6"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="001B6B73"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="001B6B73"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="000B2A4A"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00C9D3DB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="30"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <i val="1"/>
+      <color rgb="00C9D3DB"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="001B6B73"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="000B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <color rgb="002B2B2B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="001B6B73"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <color rgb="005B6B78"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <color rgb="00C9D3DB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Abadi"/>
       <b val="1"/>
       <color rgb="00C9A227"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="26"/>
+      <color rgb="001B6B73"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="00C9D3DB"/>
+      <name val="Abadi"/>
+      <color rgb="000B2A4A"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001B6B73"/>
+      <name val="Abadi"/>
+      <color theme="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C9A227"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="002B2B2B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="005B6B78"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="008A97A3"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -151,7 +205,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -262,14 +316,28 @@
       </bottom>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="00C9A227"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9A227"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A227"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9A227"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thick">
         <color rgb="00C9A227"/>
       </top>
     </border>
     <border>
-      <top style="thin">
-        <color rgb="00C9A227"/>
-      </top>
+      <bottom style="thin">
+        <color rgb="00C9D3DB"/>
+      </bottom>
     </border>
     <border>
       <right/>
@@ -470,90 +538,131 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="25" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -657,7 +766,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Formato'!A13</f>
+              <f>'FORMATO'!A13</f>
             </strRef>
           </tx>
           <spPr>
@@ -673,12 +782,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Formato'!$B$7:$M$7</f>
+              <f>'FORMATO'!$B$7:$M$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Formato'!$B$13:$M$13</f>
+              <f>'FORMATO'!$B$13:$M$13</f>
             </numRef>
           </val>
         </ser>
@@ -687,7 +796,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Formato'!A23</f>
+              <f>'FORMATO'!A23</f>
             </strRef>
           </tx>
           <spPr>
@@ -703,12 +812,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Formato'!$B$7:$M$7</f>
+              <f>'FORMATO'!$B$7:$M$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Formato'!$B$23:$M$23</f>
+              <f>'FORMATO'!$B$23:$M$23</f>
             </numRef>
           </val>
         </ser>
@@ -776,7 +885,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Formato'!A26</f>
+              <f>'FORMATO'!A26</f>
             </strRef>
           </tx>
           <spPr>
@@ -797,12 +906,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Formato'!$B$7:$M$7</f>
+              <f>'FORMATO'!$B$7:$M$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Formato'!$B$26:$M$26</f>
+              <f>'FORMATO'!$B$26:$M$26</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1181,22 +1290,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="88" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="8" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -1205,154 +1320,462 @@
       </c>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>VERSIÓN 2.0  ·  MÉXICO</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="1" t="n"/>
       <c r="C3" s="1" t="n"/>
       <c r="D3" s="1" t="n"/>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Flujo de efectivo anual</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-    </row>
-    <row r="5">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>FLUJO DE EFECTIVO ANUAL</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Formato administrativo editable · México</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n"/>
-    </row>
-    <row r="6">
+      <c r="G5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Formato administrativo profesional · editable · listo para imprimir</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n"/>
       <c r="B7" s="1" t="n"/>
       <c r="C7" s="1" t="n"/>
       <c r="D7" s="1" t="n"/>
-    </row>
-    <row r="8" ht="6" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="4" customHeight="1">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>FÓRMULAS AUTOMÁTICAS</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>LISTAS DESPLEGABLES</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>HOJAS PROTEGIDAS</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>LISTO PARA IMPRIMIR</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+    </row>
+    <row r="13" ht="6" customHeight="1">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>¿QUÉ INCLUYE ESTE ARCHIVO?</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>FORMATO</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Hoja principal de captura. Aquí registras tu información; las celdas grises calculan solas.</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>RESUMEN</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Tablero con indicadores y gráficas que se actualizan automáticamente con tus datos.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>AYUDA</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Preguntas frecuentes, glosario y lista de verificación para cerrar tu periodo.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>CÓMO USARLO</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="21" customHeight="1">
-      <c r="B11" s="7" t="n">
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="21" customHeight="1">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>Captura el saldo inicial del año.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="21" customHeight="1">
-      <c r="B12" s="7" t="n">
+      <c r="G21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="21" customHeight="1">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>Llena en las celdas de captura los ingresos y egresos esperados (o reales) de cada mes.</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="21" customHeight="1">
-      <c r="B13" s="7" t="n">
+      <c r="G22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>Puedes renombrar los conceptos de la columna A según tu negocio.</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="B14" s="7" t="n">
+      <c r="G23" s="4" t="n"/>
+    </row>
+    <row r="24" ht="21" customHeight="1">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>El flujo neto y el saldo acumulado se actualizan solos; un saldo negativo indica falta de liquidez.</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="B15" s="7" t="n">
+      <c r="G24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Personaliza: en el recuadro punteado de la esquina superior derecha inserta tu logo (Insertar &gt; Imágenes) y captura los datos de tu empresa en las celdas de captura.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>LEYENDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="9" t="inlineStr"/>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Celda de captura: escribe aquí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="11" t="inlineStr"/>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Cálculo automático: no la modifiques.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="12" t="inlineStr"/>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Encabezados y títulos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>GRUPO CANVILLE · Formatos administrativos · v1.0</t>
-        </is>
-      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Personaliza: inserta tu logotipo en el recuadro punteado de la esquina superior derecha (Insertar &gt; Imágenes) y captura los datos de tu empresa en las celdas de captura.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>RECOMENDACIONES DE USO</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="4" t="n"/>
+    </row>
+    <row r="28" ht="21" customHeight="1">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Captura primero la proyección del año y después compárala mes a mes con lo real.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="21" customHeight="1">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Un flujo neto negativo sostenido es señal para renegociar plazos con proveedores o acelerar la cobranza.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n"/>
+    </row>
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Considera los meses de pago de impuestos, aguinaldo y vacaciones: concentran salidas importantes.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="21" customHeight="1">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Revisa el saldo acumulado: debe mantenerse positivo todo el año.</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>LEYENDA DE COLORES</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="17" t="inlineStr"/>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>CELDA DE CAPTURA: escribe aquí.</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="19" t="inlineStr"/>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>CÁLCULO AUTOMÁTICO: no la modifiques.</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="20" t="inlineStr"/>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>ENCABEZADOS Y TÍTULOS.</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>GRUPO CANVILLE  ·  Formatos administrativos  ·  Para uso interno de tu empresa</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="16">
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="B4:F5"/>
+    <mergeCell ref="C28:F28"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
@@ -1385,931 +1808,1016 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>FLUJO DE EFECTIVO ANUAL</t>
         </is>
       </c>
-      <c r="M1" s="38" t="inlineStr">
+      <c r="M1" s="53" t="inlineStr">
         <is>
           <t>INSERTE SU LOGO
 (clic derecho &gt; Insertar imagen)</t>
         </is>
       </c>
-      <c r="N1" s="39" t="n"/>
+      <c r="N1" s="54" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="55" t="inlineStr">
         <is>
           <t>Proyección y control mensual</t>
         </is>
       </c>
-      <c r="B2" s="19" t="n"/>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="19" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="n"/>
-      <c r="I2" s="19" t="n"/>
-      <c r="J2" s="19" t="n"/>
-      <c r="K2" s="19" t="n"/>
-      <c r="L2" s="19" t="n"/>
-      <c r="M2" s="41" t="n"/>
-      <c r="N2" s="42" t="n"/>
+      <c r="B2" s="56" t="n"/>
+      <c r="C2" s="56" t="n"/>
+      <c r="D2" s="56" t="n"/>
+      <c r="E2" s="56" t="n"/>
+      <c r="F2" s="56" t="n"/>
+      <c r="G2" s="56" t="n"/>
+      <c r="H2" s="56" t="n"/>
+      <c r="I2" s="56" t="n"/>
+      <c r="J2" s="56" t="n"/>
+      <c r="K2" s="56" t="n"/>
+      <c r="L2" s="56" t="n"/>
+      <c r="M2" s="57" t="n"/>
+      <c r="N2" s="58" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
-        <is>
-          <t>Empresa</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Comercializadora Ejemplo S.A. de C.V.</t>
-        </is>
-      </c>
-      <c r="C4" s="43" t="n"/>
-      <c r="D4" s="44" t="n"/>
-      <c r="F4" s="22" t="inlineStr">
-        <is>
-          <t>Año</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="n">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>EMPRESA</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>COMERCIALIZADORA EJEMPLO S.A. DE C.V.</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="n"/>
+      <c r="D4" s="60" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>AÑO</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="n">
         <v>2026</v>
       </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>Saldo inicial del año</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>SALDO INICIAL DEL AÑO</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="n">
         <v>50000</v>
       </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Ene</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="inlineStr">
-        <is>
-          <t>Abr</t>
-        </is>
-      </c>
-      <c r="F7" s="24" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="G7" s="24" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>Jul</t>
-        </is>
-      </c>
-      <c r="I7" s="24" t="inlineStr">
-        <is>
-          <t>Ago</t>
-        </is>
-      </c>
-      <c r="J7" s="24" t="inlineStr">
-        <is>
-          <t>Sep</t>
-        </is>
-      </c>
-      <c r="K7" s="24" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L7" s="24" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="M7" s="24" t="inlineStr">
-        <is>
-          <t>Dic</t>
-        </is>
-      </c>
-      <c r="N7" s="24" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>ENE</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>FEB</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>ABR</t>
+        </is>
+      </c>
+      <c r="F7" s="31" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>JUN</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="I7" s="31" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="K7" s="31" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="L7" s="31" t="inlineStr">
+        <is>
+          <t>NOV</t>
+        </is>
+      </c>
+      <c r="M7" s="31" t="inlineStr">
+        <is>
+          <t>DIC</t>
+        </is>
+      </c>
+      <c r="N7" s="31" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>INGRESOS</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
-      <c r="D8" s="26" t="n"/>
-      <c r="E8" s="26" t="n"/>
-      <c r="F8" s="26" t="n"/>
-      <c r="G8" s="26" t="n"/>
-      <c r="H8" s="26" t="n"/>
-      <c r="I8" s="26" t="n"/>
-      <c r="J8" s="26" t="n"/>
-      <c r="K8" s="26" t="n"/>
-      <c r="L8" s="26" t="n"/>
-      <c r="M8" s="26" t="n"/>
-      <c r="N8" s="26" t="n"/>
+      <c r="B8" s="33" t="n"/>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="33" t="n"/>
+      <c r="I8" s="33" t="n"/>
+      <c r="J8" s="33" t="n"/>
+      <c r="K8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="33" t="n"/>
+      <c r="N8" s="33" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
-        <is>
-          <t>Ventas de contado</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="n">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t>VENTAS DE CONTADO</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
         <v>109250</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="30" t="n">
         <v>126500</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="30" t="n">
         <v>138000</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="30" t="n">
         <v>120750</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="30" t="n">
         <v>149500</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="30" t="n">
         <v>161000</v>
       </c>
-      <c r="H9" s="23" t="n">
+      <c r="H9" s="30" t="n">
         <v>143750</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="30" t="n">
         <v>155250</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="30" t="n">
         <v>172500</v>
       </c>
-      <c r="K9" s="23" t="n">
+      <c r="K9" s="30" t="n">
         <v>166750</v>
       </c>
-      <c r="L9" s="23" t="n">
+      <c r="L9" s="30" t="n">
         <v>184000</v>
       </c>
-      <c r="M9" s="23" t="n">
+      <c r="M9" s="30" t="n">
         <v>207000</v>
       </c>
-      <c r="N9" s="28">
+      <c r="N9" s="35">
         <f>SUM(B9:M9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>Cobranza de crédito</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="n">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>COBRANZA DE CRÉDITO</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n">
         <v>69000</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="30" t="n">
         <v>74750</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="30" t="n">
         <v>80500</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="30" t="n">
         <v>82800</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="30" t="n">
         <v>86250</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="30" t="n">
         <v>92000</v>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H10" s="30" t="n">
         <v>89700</v>
       </c>
-      <c r="I10" s="23" t="n">
+      <c r="I10" s="30" t="n">
         <v>94300</v>
       </c>
-      <c r="J10" s="23" t="n">
+      <c r="J10" s="30" t="n">
         <v>103500</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="30" t="n">
         <v>101200</v>
       </c>
-      <c r="L10" s="23" t="n">
+      <c r="L10" s="30" t="n">
         <v>109250</v>
       </c>
-      <c r="M10" s="23" t="n">
+      <c r="M10" s="30" t="n">
         <v>115000</v>
       </c>
-      <c r="N10" s="28">
+      <c r="N10" s="35">
         <f>SUM(B10:M10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="n">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="n">
         <v>23000</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="30" t="n">
         <v>20700</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="30" t="n">
         <v>28750</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="30" t="n">
         <v>25300</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="30" t="n">
         <v>32200</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="30" t="n">
         <v>34500</v>
       </c>
-      <c r="H11" s="23" t="n">
+      <c r="H11" s="30" t="n">
         <v>29900</v>
       </c>
-      <c r="I11" s="23" t="n">
+      <c r="I11" s="30" t="n">
         <v>36800</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="30" t="n">
         <v>40250</v>
       </c>
-      <c r="K11" s="23" t="n">
+      <c r="K11" s="30" t="n">
         <v>37950</v>
       </c>
-      <c r="L11" s="23" t="n">
+      <c r="L11" s="30" t="n">
         <v>43700</v>
       </c>
-      <c r="M11" s="23" t="n">
+      <c r="M11" s="30" t="n">
         <v>51750</v>
       </c>
-      <c r="N11" s="28">
+      <c r="N11" s="35">
         <f>SUM(B11:M11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>Otros ingresos</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="n">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>OTROS INGRESOS</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="n">
         <v>3450</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="30" t="n">
         <v>2300</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="30" t="n">
         <v>4600</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="30" t="n">
         <v>3450</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="30" t="n">
         <v>5750</v>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G12" s="30" t="n">
         <v>4600</v>
       </c>
-      <c r="H12" s="23" t="n">
+      <c r="H12" s="30" t="n">
         <v>3450</v>
       </c>
-      <c r="I12" s="23" t="n">
+      <c r="I12" s="30" t="n">
         <v>6900</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J12" s="30" t="n">
         <v>5750</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="K12" s="30" t="n">
         <v>4600</v>
       </c>
-      <c r="L12" s="23" t="n">
+      <c r="L12" s="30" t="n">
         <v>6900</v>
       </c>
-      <c r="M12" s="23" t="n">
+      <c r="M12" s="30" t="n">
         <v>9200</v>
       </c>
-      <c r="N12" s="28">
+      <c r="N12" s="35">
         <f>SUM(B12:M12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Total ingresos</t>
-        </is>
-      </c>
-      <c r="B13" s="28">
+      <c r="A13" s="36" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+      <c r="B13" s="35">
         <f>SUM(B9:B12)</f>
         <v/>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="35">
         <f>SUM(C9:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="35">
         <f>SUM(D9:D12)</f>
         <v/>
       </c>
-      <c r="E13" s="28">
+      <c r="E13" s="35">
         <f>SUM(E9:E12)</f>
         <v/>
       </c>
-      <c r="F13" s="28">
+      <c r="F13" s="35">
         <f>SUM(F9:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="28">
+      <c r="G13" s="35">
         <f>SUM(G9:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="35">
         <f>SUM(H9:H12)</f>
         <v/>
       </c>
-      <c r="I13" s="28">
+      <c r="I13" s="35">
         <f>SUM(I9:I12)</f>
         <v/>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="35">
         <f>SUM(J9:J12)</f>
         <v/>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="35">
         <f>SUM(K9:K12)</f>
         <v/>
       </c>
-      <c r="L13" s="28">
+      <c r="L13" s="35">
         <f>SUM(L9:L12)</f>
         <v/>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="35">
         <f>SUM(M9:M12)</f>
         <v/>
       </c>
-      <c r="N13" s="28">
+      <c r="N13" s="35">
         <f>SUM(N9:N12)</f>
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="n"/>
+      <c r="N14" s="4" t="n"/>
+    </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>EGRESOS</t>
         </is>
       </c>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="26" t="n"/>
-      <c r="D15" s="26" t="n"/>
-      <c r="E15" s="26" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="26" t="n"/>
-      <c r="H15" s="26" t="n"/>
-      <c r="I15" s="26" t="n"/>
-      <c r="J15" s="26" t="n"/>
-      <c r="K15" s="26" t="n"/>
-      <c r="L15" s="26" t="n"/>
-      <c r="M15" s="26" t="n"/>
-      <c r="N15" s="26" t="n"/>
+      <c r="B15" s="33" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="33" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="33" t="n"/>
+      <c r="L15" s="33" t="n"/>
+      <c r="M15" s="33" t="n"/>
+      <c r="N15" s="33" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
-        <is>
-          <t>Nómina y cargas sociales</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="n">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>NÓMINA Y CARGAS SOCIALES</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
         <v>70000</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="30" t="n">
         <v>70000</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="30" t="n">
         <v>72000</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="30" t="n">
         <v>72000</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="30" t="n">
         <v>74000</v>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="30" t="n">
         <v>74000</v>
       </c>
-      <c r="H16" s="23" t="n">
+      <c r="H16" s="30" t="n">
         <v>76000</v>
       </c>
-      <c r="I16" s="23" t="n">
+      <c r="I16" s="30" t="n">
         <v>76000</v>
       </c>
-      <c r="J16" s="23" t="n">
+      <c r="J16" s="30" t="n">
         <v>78000</v>
       </c>
-      <c r="K16" s="23" t="n">
+      <c r="K16" s="30" t="n">
         <v>78000</v>
       </c>
-      <c r="L16" s="23" t="n">
+      <c r="L16" s="30" t="n">
         <v>80000</v>
       </c>
-      <c r="M16" s="23" t="n">
+      <c r="M16" s="30" t="n">
         <v>95000</v>
       </c>
-      <c r="N16" s="28">
+      <c r="N16" s="35">
         <f>SUM(B16:M16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>Renta</t>
-        </is>
-      </c>
-      <c r="B17" s="23" t="n">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>RENTA</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="H17" s="23" t="n">
+      <c r="H17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="I17" s="23" t="n">
+      <c r="I17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="J17" s="23" t="n">
+      <c r="J17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="K17" s="23" t="n">
+      <c r="K17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="L17" s="23" t="n">
+      <c r="L17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="M17" s="23" t="n">
+      <c r="M17" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="N17" s="28">
+      <c r="N17" s="35">
         <f>SUM(B17:M17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Proveedores</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="n">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>PROVEEDORES</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
         <v>80000</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="30" t="n">
         <v>85000</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="30" t="n">
         <v>92000</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="30" t="n">
         <v>88000</v>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="30" t="n">
         <v>98000</v>
       </c>
-      <c r="G18" s="23" t="n">
+      <c r="G18" s="30" t="n">
         <v>105000</v>
       </c>
-      <c r="H18" s="23" t="n">
+      <c r="H18" s="30" t="n">
         <v>96000</v>
       </c>
-      <c r="I18" s="23" t="n">
+      <c r="I18" s="30" t="n">
         <v>104000</v>
       </c>
-      <c r="J18" s="23" t="n">
+      <c r="J18" s="30" t="n">
         <v>112000</v>
       </c>
-      <c r="K18" s="23" t="n">
+      <c r="K18" s="30" t="n">
         <v>108000</v>
       </c>
-      <c r="L18" s="23" t="n">
+      <c r="L18" s="30" t="n">
         <v>118000</v>
       </c>
-      <c r="M18" s="23" t="n">
+      <c r="M18" s="30" t="n">
         <v>130000</v>
       </c>
-      <c r="N18" s="28">
+      <c r="N18" s="35">
         <f>SUM(B18:M18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
-        <is>
-          <t>Servicios (luz, agua, internet)</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="n">
+      <c r="A19" s="34" t="inlineStr">
+        <is>
+          <t>SERVICIOS (LUZ, AGUA, INTERNET)</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="n">
         <v>9000</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="30" t="n">
         <v>9000</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="30" t="n">
         <v>9000</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="H19" s="23" t="n">
+      <c r="H19" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="I19" s="23" t="n">
+      <c r="I19" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="J19" s="23" t="n">
+      <c r="J19" s="30" t="n">
         <v>11000</v>
       </c>
-      <c r="K19" s="23" t="n">
+      <c r="K19" s="30" t="n">
         <v>11000</v>
       </c>
-      <c r="L19" s="23" t="n">
+      <c r="L19" s="30" t="n">
         <v>11000</v>
       </c>
-      <c r="M19" s="23" t="n">
+      <c r="M19" s="30" t="n">
         <v>11000</v>
       </c>
-      <c r="N19" s="28">
+      <c r="N19" s="35">
         <f>SUM(B19:M19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
-        <is>
-          <t>Impuestos (IVA/ISR)</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="n">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>IMPUESTOS (IVA/ISR)</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="n">
         <v>18000</v>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="30" t="n">
         <v>20000</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="30" t="n">
         <v>22000</v>
       </c>
-      <c r="F20" s="23" t="n">
+      <c r="F20" s="30" t="n">
         <v>26000</v>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="30" t="n">
         <v>28000</v>
       </c>
-      <c r="H20" s="23" t="n">
+      <c r="H20" s="30" t="n">
         <v>25000</v>
       </c>
-      <c r="I20" s="23" t="n">
+      <c r="I20" s="30" t="n">
         <v>28000</v>
       </c>
-      <c r="J20" s="23" t="n">
+      <c r="J20" s="30" t="n">
         <v>32000</v>
       </c>
-      <c r="K20" s="23" t="n">
+      <c r="K20" s="30" t="n">
         <v>30000</v>
       </c>
-      <c r="L20" s="23" t="n">
+      <c r="L20" s="30" t="n">
         <v>34000</v>
       </c>
-      <c r="M20" s="23" t="n">
+      <c r="M20" s="30" t="n">
         <v>40000</v>
       </c>
-      <c r="N20" s="28">
+      <c r="N20" s="35">
         <f>SUM(B20:M20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>Publicidad</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="n">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>PUBLICIDAD</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="H21" s="23" t="n">
+      <c r="H21" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="I21" s="23" t="n">
+      <c r="I21" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="J21" s="23" t="n">
+      <c r="J21" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="K21" s="23" t="n">
+      <c r="K21" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="L21" s="23" t="n">
+      <c r="L21" s="30" t="n">
         <v>10000</v>
       </c>
-      <c r="M21" s="23" t="n">
+      <c r="M21" s="30" t="n">
         <v>14000</v>
       </c>
-      <c r="N21" s="28">
+      <c r="N21" s="35">
         <f>SUM(B21:M21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
-        <is>
-          <t>Otros egresos</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="n">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>OTROS EGRESOS</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="n">
         <v>5000</v>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="30" t="n">
         <v>4000</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="30" t="n">
         <v>5000</v>
       </c>
-      <c r="F22" s="23" t="n">
+      <c r="F22" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="30" t="n">
         <v>7000</v>
       </c>
-      <c r="H22" s="23" t="n">
+      <c r="H22" s="30" t="n">
         <v>5000</v>
       </c>
-      <c r="I22" s="23" t="n">
+      <c r="I22" s="30" t="n">
         <v>7000</v>
       </c>
-      <c r="J22" s="23" t="n">
+      <c r="J22" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="K22" s="23" t="n">
+      <c r="K22" s="30" t="n">
         <v>6000</v>
       </c>
-      <c r="L22" s="23" t="n">
+      <c r="L22" s="30" t="n">
         <v>8000</v>
       </c>
-      <c r="M22" s="23" t="n">
+      <c r="M22" s="30" t="n">
         <v>9000</v>
       </c>
-      <c r="N22" s="28">
+      <c r="N22" s="35">
         <f>SUM(B22:M22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>Total egresos</t>
-        </is>
-      </c>
-      <c r="B23" s="28">
+      <c r="A23" s="36" t="inlineStr">
+        <is>
+          <t>TOTAL EGRESOS</t>
+        </is>
+      </c>
+      <c r="B23" s="35">
         <f>SUM(B16:B22)</f>
         <v/>
       </c>
-      <c r="C23" s="28">
+      <c r="C23" s="35">
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="35">
         <f>SUM(D16:D22)</f>
         <v/>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="35">
         <f>SUM(E16:E22)</f>
         <v/>
       </c>
-      <c r="F23" s="28">
+      <c r="F23" s="35">
         <f>SUM(F16:F22)</f>
         <v/>
       </c>
-      <c r="G23" s="28">
+      <c r="G23" s="35">
         <f>SUM(G16:G22)</f>
         <v/>
       </c>
-      <c r="H23" s="28">
+      <c r="H23" s="35">
         <f>SUM(H16:H22)</f>
         <v/>
       </c>
-      <c r="I23" s="28">
+      <c r="I23" s="35">
         <f>SUM(I16:I22)</f>
         <v/>
       </c>
-      <c r="J23" s="28">
+      <c r="J23" s="35">
         <f>SUM(J16:J22)</f>
         <v/>
       </c>
-      <c r="K23" s="28">
+      <c r="K23" s="35">
         <f>SUM(K16:K22)</f>
         <v/>
       </c>
-      <c r="L23" s="28">
+      <c r="L23" s="35">
         <f>SUM(L16:L22)</f>
         <v/>
       </c>
-      <c r="M23" s="28">
+      <c r="M23" s="35">
         <f>SUM(M16:M22)</f>
         <v/>
       </c>
-      <c r="N23" s="28">
+      <c r="N23" s="35">
         <f>SUM(N16:N22)</f>
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="n"/>
+    </row>
     <row r="25">
-      <c r="A25" s="29" t="inlineStr">
+      <c r="A25" s="36" t="inlineStr">
         <is>
           <t>FLUJO NETO DEL MES</t>
         </is>
       </c>
-      <c r="B25" s="30">
+      <c r="B25" s="37">
         <f>B13-B23</f>
         <v/>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="37">
         <f>C13-C23</f>
         <v/>
       </c>
-      <c r="D25" s="30">
+      <c r="D25" s="37">
         <f>D13-D23</f>
         <v/>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="37">
         <f>E13-E23</f>
         <v/>
       </c>
-      <c r="F25" s="30">
+      <c r="F25" s="37">
         <f>F13-F23</f>
         <v/>
       </c>
-      <c r="G25" s="30">
+      <c r="G25" s="37">
         <f>G13-G23</f>
         <v/>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="37">
         <f>H13-H23</f>
         <v/>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="37">
         <f>I13-I23</f>
         <v/>
       </c>
-      <c r="J25" s="30">
+      <c r="J25" s="37">
         <f>J13-J23</f>
         <v/>
       </c>
-      <c r="K25" s="30">
+      <c r="K25" s="37">
         <f>K13-K23</f>
         <v/>
       </c>
-      <c r="L25" s="30">
+      <c r="L25" s="37">
         <f>L13-L23</f>
         <v/>
       </c>
-      <c r="M25" s="30">
+      <c r="M25" s="37">
         <f>M13-M23</f>
         <v/>
       </c>
-      <c r="N25" s="31">
+      <c r="N25" s="38">
         <f>SUM(B25:M25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="36" t="inlineStr">
         <is>
           <t>SALDO FINAL ACUMULADO</t>
         </is>
       </c>
-      <c r="B26" s="30">
+      <c r="B26" s="37">
         <f>$B$5+B25</f>
         <v/>
       </c>
-      <c r="C26" s="30">
+      <c r="C26" s="37">
         <f>B26+C25</f>
         <v/>
       </c>
-      <c r="D26" s="30">
+      <c r="D26" s="37">
         <f>C26+D25</f>
         <v/>
       </c>
-      <c r="E26" s="30">
+      <c r="E26" s="37">
         <f>D26+E25</f>
         <v/>
       </c>
-      <c r="F26" s="30">
+      <c r="F26" s="37">
         <f>E26+F25</f>
         <v/>
       </c>
-      <c r="G26" s="30">
+      <c r="G26" s="37">
         <f>F26+G25</f>
         <v/>
       </c>
-      <c r="H26" s="30">
+      <c r="H26" s="37">
         <f>G26+H25</f>
         <v/>
       </c>
-      <c r="I26" s="30">
+      <c r="I26" s="37">
         <f>H26+I25</f>
         <v/>
       </c>
-      <c r="J26" s="30">
+      <c r="J26" s="37">
         <f>I26+J25</f>
         <v/>
       </c>
-      <c r="K26" s="30">
+      <c r="K26" s="37">
         <f>J26+K25</f>
         <v/>
       </c>
-      <c r="L26" s="30">
+      <c r="L26" s="37">
         <f>K26+L25</f>
         <v/>
       </c>
-      <c r="M26" s="30">
+      <c r="M26" s="37">
         <f>L26+M25</f>
         <v/>
       </c>
+      <c r="N26" s="4" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
@@ -2356,83 +2864,99 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>RESUMEN DE FLUJO DE EFECTIVO</t>
         </is>
       </c>
-      <c r="H1" s="38" t="inlineStr">
+      <c r="H1" s="53" t="inlineStr">
         <is>
           <t>INSERTE SU LOGO
 (clic derecho &gt; Insertar imagen)</t>
         </is>
       </c>
-      <c r="I1" s="45" t="n"/>
-      <c r="J1" s="39" t="n"/>
+      <c r="I1" s="61" t="n"/>
+      <c r="J1" s="54" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="55" t="inlineStr">
         <is>
           <t>Ingresos, egresos y saldo acumulado por mes</t>
         </is>
       </c>
-      <c r="B2" s="19" t="n"/>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="19" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="41" t="n"/>
-      <c r="I2" s="46" t="n"/>
-      <c r="J2" s="42" t="n"/>
+      <c r="B2" s="56" t="n"/>
+      <c r="C2" s="56" t="n"/>
+      <c r="D2" s="56" t="n"/>
+      <c r="E2" s="56" t="n"/>
+      <c r="F2" s="56" t="n"/>
+      <c r="G2" s="56" t="n"/>
+      <c r="H2" s="57" t="n"/>
+      <c r="I2" s="62" t="n"/>
+      <c r="J2" s="58" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="47" t="inlineStr">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>INGRESOS DEL AÑO</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n"/>
-      <c r="D4" s="47" t="inlineStr">
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="63" t="inlineStr">
         <is>
           <t>EGRESOS DEL AÑO</t>
         </is>
       </c>
-      <c r="E4" s="48" t="n"/>
-      <c r="F4" s="47" t="inlineStr">
+      <c r="E4" s="64" t="n"/>
+      <c r="F4" s="63" t="inlineStr">
         <is>
           <t>FLUJO NETO</t>
         </is>
       </c>
-      <c r="G4" s="48" t="n"/>
-      <c r="H4" s="47" t="inlineStr">
+      <c r="G4" s="64" t="n"/>
+      <c r="H4" s="63" t="inlineStr">
         <is>
           <t>SALDO FINAL</t>
         </is>
       </c>
-      <c r="I4" s="48" t="n"/>
+      <c r="I4" s="64" t="n"/>
+      <c r="J4" s="4" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="B5" s="49">
-        <f>Formato!N13</f>
-        <v/>
-      </c>
-      <c r="C5" s="50" t="n"/>
-      <c r="D5" s="49">
-        <f>Formato!N23</f>
-        <v/>
-      </c>
-      <c r="E5" s="50" t="n"/>
-      <c r="F5" s="49">
-        <f>Formato!N25</f>
-        <v/>
-      </c>
-      <c r="G5" s="50" t="n"/>
-      <c r="H5" s="49">
-        <f>Formato!M26</f>
-        <v/>
-      </c>
-      <c r="I5" s="50" t="n"/>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="65">
+        <f>FORMATO!N13</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="n"/>
+      <c r="D5" s="65">
+        <f>FORMATO!N23</f>
+        <v/>
+      </c>
+      <c r="E5" s="66" t="n"/>
+      <c r="F5" s="65">
+        <f>FORMATO!N25</f>
+        <v/>
+      </c>
+      <c r="G5" s="66" t="n"/>
+      <c r="H5" s="65">
+        <f>FORMATO!M26</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="n"/>
+      <c r="J5" s="4" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
@@ -2462,4 +2986,341 @@
   </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B6B73"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="45" t="inlineStr">
+        <is>
+          <t>AYUDA Y PREGUNTAS FRECUENTES</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="46" t="inlineStr">
+        <is>
+          <t>FLUJO DE EFECTIVO ANUAL</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>PREGUNTAS FRECUENTES</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>¿Debo incluir el IVA?</t>
+        </is>
+      </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>Sí, el flujo de efectivo refleja el dinero real que entra y sale, con impuestos incluidos.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>¿Puedo cambiar los conceptos?</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>Sí, edita los nombres de la columna A; las fórmulas no se alteran.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="53" customHeight="1">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>¿Por qué no puedo escribir en algunas celdas?</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>La hoja está protegida para que no se borren fórmulas por accidente. Solo se editan las celdas de captura (color crema). Si necesitas modificar algo más: pestaña Revisar &gt; Desproteger hoja (no tiene contraseña).</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>¿Cómo agrego mi logotipo?</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>Haz clic en el recuadro punteado de la esquina superior derecha del formato y usa Insertar &gt; Imágenes. Ajusta el tamaño sin salirte del recuadro.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>¿Cómo lo imprimo o lo convierto a PDF?</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>Archivo &gt; Imprimir (ya está ajustado a una hoja de ancho). Para PDF elige 'Microsoft Print to PDF' o Archivo &gt; Exportar &gt; PDF.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t>¿Con qué versiones de Excel funciona?</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>Excel 2016, 2019, 2021 y Microsoft 365 (Windows y Mac). Funciona en LibreOffice y Google Sheets, aunque algunas gráficas y formatos pueden verse distintos.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="47" t="inlineStr">
+        <is>
+          <t>¿Por qué la letra se ve diferente?</t>
+        </is>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>El diseño usa la fuente Abadi, incluida en Microsoft 365. Si tu versión no la tiene, Excel la sustituye por otra; no afecta el funcionamiento.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="47" t="inlineStr">
+        <is>
+          <t>¿Puedo usarlo en varias empresas o por varios años?</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>Sí. Guarda una copia del archivo por empresa o por periodo (Archivo &gt; Guardar como) y deja el original en blanco como plantilla maestra.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>GLOSARIO</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="49" t="inlineStr">
+        <is>
+          <t>FLUJO NETO</t>
+        </is>
+      </c>
+      <c r="D16" s="50" t="inlineStr">
+        <is>
+          <t>Ingresos del mes - egresos del mes.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>SALDO ACUMULADO</t>
+        </is>
+      </c>
+      <c r="D17" s="50" t="inlineStr">
+        <is>
+          <t>Saldo inicial + suma de flujos netos hasta el mes.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="49" t="inlineStr">
+        <is>
+          <t>LIQUIDEZ</t>
+        </is>
+      </c>
+      <c r="D18" s="50" t="inlineStr">
+        <is>
+          <t>Capacidad de pagar obligaciones de corto plazo.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>LISTA DE VERIFICACIÓN (marca ☑ al completar)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="C21" s="52" t="inlineStr">
+        <is>
+          <t>Saldo inicial capturado</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
+        <is>
+          <t>Ingresos esperados por mes capturados</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
+        <is>
+          <t>Egresos fijos y variables capturados</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="C24" s="52" t="inlineStr">
+        <is>
+          <t>Se revisó el mes con menor saldo</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="6">
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B21 B22 B23 B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"☐,☑"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>